<commit_message>
Updatet graph of second benchmark
</commit_message>
<xml_diff>
--- a/Documents/paper_figures/DataSequentialCutoffBenchmark.xlsx
+++ b/Documents/paper_figures/DataSequentialCutoffBenchmark.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Noah\Desktop\HSO\Seminar 1\IT-Anwendungen\Paper_ParallelArrayOperationsJava\Documents\paper_figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3DEA8F5-BFA0-455F-8E09-9A7F9C984361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C65F78FF-C97C-4F05-8E14-C975CB8A520C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFB4A8D3-EF7B-4887-A2E4-1F6328295819}"/>
   </bookViews>
@@ -126,6 +126,36 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="de-DE"/>
+              <a:t>Runtimes</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" baseline="0"/>
+              <a:t> of second benchmark</a:t>
+            </a:r>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -162,10 +192,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="8.5636482939632552E-2"/>
-          <c:y val="0.17171296296296296"/>
-          <c:w val="0.86603018372703411"/>
-          <c:h val="0.72125801983085447"/>
+          <c:x val="0.14103150710146356"/>
+          <c:y val="0.17171309930879256"/>
+          <c:w val="0.81063527151833747"/>
+          <c:h val="0.70300392819721191"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -297,6 +327,8 @@
         <c:axId val="1199671936"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="7500"/>
+          <c:min val="500"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -314,6 +346,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-DE"/>
+                  <a:t>Array size</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -354,6 +441,8 @@
         <c:crossAx val="1262384688"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
+        <c:majorUnit val="1000"/>
+        <c:minorUnit val="100"/>
       </c:valAx>
       <c:valAx>
         <c:axId val="1262384688"/>
@@ -376,6 +465,66 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-DE"/>
+                  <a:t>Average execution time</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="de-DE" baseline="0"/>
+                  <a:t> [ms]</a:t>
+                </a:r>
+                <a:endParaRPr lang="de-DE"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1023,15 +1172,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>251129</xdr:colOff>
+      <xdr:colOff>284259</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>2154</xdr:rowOff>
+      <xdr:rowOff>22032</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>65599</xdr:colOff>
+      <xdr:colOff>98729</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>2154</xdr:rowOff>
+      <xdr:rowOff>22032</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>